<commit_message>
📊 Auto scan: 2026-09-14
</commit_message>
<xml_diff>
--- a/archive/2026-09-14/report.xlsx
+++ b/archive/2026-09-14/report.xlsx
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5">
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -600,10 +600,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -664,7 +664,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>미운 우리 새끼</t>
+          <t>염경엽</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -695,31 +695,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nascar race today</t>
+          <t>사우디</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>100</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>RSS</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>14.7</v>
+      </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -745,7 +741,7 @@
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>3.58</v>
+        <v>3.74</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -753,34 +749,38 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>사우디</t>
+          <t>salma hayek</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>google</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
       <c r="E5" t="n">
         <v>100</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>14.14</v>
-      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>수혜주</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -801,17 +801,17 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>코스닥 테마주 디렉터리 — 관련주·수혜주 53개 테마 총정리 | kosdaq.xyz</t>
+          <t>오늘 테마주 대장주 순위 Top 64 — 관련주·거래대금 | Reload Kospi</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Stocks</t>
+          <t>관련주</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -832,7 +832,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Most Mentioned WSB Stocks Today (WallStreetBets Tracker)</t>
+          <t>오늘 테마주 대장주 순위 Top 64 — 관련주·거래대금 | Reload Kospi</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -842,7 +842,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>테마주</t>
+          <t>Stocks</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -863,48 +863,48 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>오늘 테마주 대장주 순위 Top 64 — 관련주·거래대금 | Reload Kospi</t>
+          <t>Most Mentioned WSB Stocks Today (WallStreetBets Tracker)</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>관련주</t>
+          <t>current events</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>google</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
       <c r="E9" t="n">
-        <v>100</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
+        <v>96</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>오늘 테마주 대장주 순위 Top 64 — 관련주·거래대금 | Reload Kospi</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>10</v>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tj hockenson</t>
+          <t>파업</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -935,12 +935,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>장인화</t>
+          <t>테마주</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -948,25 +948,25 @@
           <t>KR</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>96</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>RSS</t>
-        </is>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>오늘 테마주 대장주 순위 Top 64 — 관련주·거래대금 | Reload Kospi</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>총정리</t>
+          <t>수혜주</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -997,7 +997,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>john madden</t>
+          <t>epstein files</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1028,7 +1028,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>전소미</t>
+          <t>두산에너 빌리티</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1059,7 +1059,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>lioness season 3 how many episodes</t>
+          <t>saudi arabia</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1090,7 +1090,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>오늘날씨</t>
+          <t>오타니 쇼헤이</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1121,7 +1121,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>총정리</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1142,7 +1142,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>오늘 테마주 대장주 순위 Top 64 — 관련주·거래대금 | Reload Kospi</t>
+          <t>코스닥 테마주 디렉터리 — 관련주·수혜주 53개 테마 총정리 | kosdaq.xyz</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -1152,34 +1152,38 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>양자암호</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
-        <v>2.83</v>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ETF Launches</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>barcelona sc - delfín</t>
+          <t>iran war</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1210,7 +1214,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>김동관</t>
+          <t>임시 공휴일</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1241,7 +1245,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>광통신</t>
+          <t>양자암호</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1256,11 +1260,11 @@
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
-        <v>2.73</v>
+        <v>2.7</v>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
@@ -1268,7 +1272,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>javonte williams</t>
+          <t>조훈현</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1278,7 +1282,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1299,7 +1303,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>klasemen manchester united f.c. vs man city</t>
+          <t>king charles letter about harry and meghan</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1309,7 +1313,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1330,7 +1334,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>실시간</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1351,7 +1355,7 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>국내 주식 정보 커뮤니티 종목 토론방 추천 투자정보 전략수집 : 네이버 블로그</t>
+          <t>오늘 급등주 Top 20 — 실시간 등락률·거래량 급증 순위 | Reload Kospi</t>
         </is>
       </c>
       <c r="I24" t="n">
@@ -1361,7 +1365,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>블로그</t>
+          <t>Trending</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1371,7 +1375,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1382,7 +1386,7 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>국내 주식 정보 커뮤니티 종목 토론방 추천 투자정보 전략수집 : 네이버 블로그</t>
+          <t>Reddit Stocks: Most Mentioned &amp;amp; Trending Today | AltIndex</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -1423,12 +1427,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ETF</t>
+          <t>gma deals and steals</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>google</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1436,30 +1440,30 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="n">
+        <v>7</v>
+      </c>
       <c r="E27" t="n">
-        <v>78</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
+        <v>76</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>ETF Launches</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>6</v>
-      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>친환경선박</t>
+          <t>삼성전자 채용</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>google</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1467,26 +1471,30 @@
           <t>KR</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>7</v>
+      </c>
       <c r="E28" t="n">
         <v>76</v>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="n">
-        <v>2.55</v>
-      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>복권</t>
+          <t>친환경선박</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1494,56 +1502,48 @@
           <t>KR</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>7</v>
-      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
         <v>76</v>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>RSS</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="n">
+        <v>2.55</v>
+      </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>harrison smith</t>
+          <t>광통신</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>7</v>
-      </c>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
-        <v>76</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>RSS</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
+        <v>75</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="n">
+        <v>2.52</v>
+      </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>jennifer garner</t>
+          <t>프리시전 캐스트파츠</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1574,7 +1574,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>해군</t>
+          <t>mrvl stock</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1605,44 +1605,48 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>소형원자로</t>
+          <t>ETFs</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>New ETFs - ETF Trends</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Trending</t>
+          <t>소형원자로</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1650,20 +1654,16 @@
         <v>70</v>
       </c>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Ape Wisdom | Trending Stocks on r/wallstreetbets</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>5</v>
-      </c>
+      <c r="G34" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>대장주</t>
+          <t>이재명</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1684,7 +1684,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>오늘 테마주 대장주 순위 Top 64 — 관련주·거래대금 | Reload Kospi</t>
+          <t>이재명 관련주 - 정책 수혜주 Top 10 총정리 (2025 최신판)</t>
         </is>
       </c>
       <c r="I35" t="n">
@@ -1694,7 +1694,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>이재명</t>
+          <t>블로그</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1715,7 +1715,7 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>이재명 관련주 - 정책 수혜주 Top 10 총정리 (2025 최신판)</t>
+          <t>국내 주식 정보 커뮤니티 종목 토론방 추천 투자정보 전략수집 : 네이버 블로그</t>
         </is>
       </c>
       <c r="I36" t="n">
@@ -1725,12 +1725,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>로베르토 데 제르비</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1738,30 +1738,30 @@
           <t>KR</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>9</v>
-      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>68</v>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>RSS</t>
-        </is>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>국내 주식 정보 커뮤니티 종목 토론방 추천 투자정보 전략수집 : 네이버 블로그</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>michael taaffe</t>
+          <t>amp</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1769,52 +1769,56 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>9</v>
-      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>68</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>RSS</t>
-        </is>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Reddit Stocks: Most Mentioned &amp;amp; Trending Today | AltIndex</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>원전</t>
+          <t>the pitt</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>google</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>9</v>
+      </c>
       <c r="E39" t="n">
-        <v>66</v>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="n">
-        <v>2.23</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>황신혜</t>
+          <t>박주호</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1828,10 +1832,10 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E40" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -1845,7 +1849,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>latest trump news cnn</t>
+          <t>oasis</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1876,69 +1880,65 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mentioned</t>
+          <t>갤러리아백화점</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>google</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>10</v>
+      </c>
       <c r="E42" t="n">
-        <v>62</v>
-      </c>
-      <c r="F42" t="inlineStr"/>
+        <v>64</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Most Mentioned WSB Stocks Today (WallStreetBets Tracker)</t>
-        </is>
-      </c>
-      <c r="I42" t="n">
-        <v>4</v>
-      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Most</t>
+          <t>원전</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Most Mentioned WSB Stocks Today (WallStreetBets Tracker)</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>4</v>
-      </c>
+      <c r="G43" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>오늘의</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1969,7 +1969,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Week</t>
+          <t>Mentioned</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1990,7 +1990,7 @@
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>This Week&amp;#x27;s Best Performing Stocks, Sectors, Industries Rankings ...</t>
+          <t>Most Mentioned WSB Stocks Today (WallStreetBets Tracker)</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -2000,7 +2000,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Best</t>
+          <t>New</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2021,7 +2021,7 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>This Week&amp;#x27;s Best Performing Stocks, Sectors, Industries Rankings ...</t>
+          <t>New ETFs - ETF Trends</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -2031,7 +2031,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ETFs</t>
+          <t>대장주</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -2052,7 +2052,7 @@
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>7 Best Thematic ETFs to Buy in 2026 | Investing | U.S. News</t>
+          <t>오늘 테마주 대장주 순위 Top 64 — 관련주·거래대금 | Reload Kospi</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -2062,7 +2062,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>wallstreetbets</t>
+          <t>Most</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2083,7 +2083,7 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Ape Wisdom | Trending Stocks on r/wallstreetbets</t>
+          <t>Most Mentioned WSB Stocks Today (WallStreetBets Tracker)</t>
         </is>
       </c>
       <c r="I48" t="n">
@@ -2093,12 +2093,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>원자력</t>
+          <t>오늘의</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2108,19 +2108,23 @@
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F49" t="inlineStr"/>
-      <c r="G49" t="n">
-        <v>2.01</v>
-      </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>오늘의 국내주식 테마 — 코스피·코스닥 섹터별 테마주 · 업종 | Kostock</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>발사체</t>
+          <t>AI 전력</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2135,11 +2139,11 @@
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="n">
-        <v>1.97</v>
+        <v>1.9</v>
       </c>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
@@ -2147,7 +2151,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AI 전력</t>
+          <t>원자력</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2162,11 +2166,11 @@
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="n">
-        <v>1.9</v>
+        <v>1.86</v>
       </c>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
@@ -2205,12 +2209,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Kospi</t>
+          <t>발사체</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2223,20 +2227,16 @@
         <v>54</v>
       </c>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>오늘 테마주 대장주 순위 Top 64 — 관련주·거래대금 | Reload Kospi</t>
-        </is>
-      </c>
-      <c r="I53" t="n">
-        <v>3</v>
-      </c>
+      <c r="G53" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>코스피</t>
+          <t>Kospi</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2257,7 +2257,7 @@
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>오늘의 국내주식 테마 — 코스피·코스닥 섹터별 테마주 · 업종 | Kostock</t>
+          <t>오늘 테마주 대장주 순위 Top 64 — 관련주·거래대금 | Reload Kospi</t>
         </is>
       </c>
       <c r="I54" t="n">
@@ -2267,7 +2267,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>국내주식</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2298,7 +2298,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>실시간</t>
+          <t>코스피</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2319,7 +2319,7 @@
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>오늘 급등주 실시간 — 등락률·거래량 급증 순위 | Reload Kospi</t>
+          <t>오늘의 국내주식 테마 — 코스피·코스닥 섹터별 테마주 · 업종 | Kostock</t>
         </is>
       </c>
       <c r="I56" t="n">
@@ -2329,7 +2329,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>전력기기</t>
+          <t>테슬라봇</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2356,7 +2356,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>산업용 로봇</t>
+          <t>분리막</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2371,68 +2371,14 @@
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="n">
-        <v>1.55</v>
+        <v>1.53</v>
       </c>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>AI 가속기</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>naver</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="n">
-        <v>45</v>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>분리막</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>naver</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="n">
-        <v>45</v>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9099,7 +9045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9113,7 +9059,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="41" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -9209,7 +9155,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>64.40000000000001</v>
+        <v>63.5</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -9220,7 +9166,7 @@
         <v>60</v>
       </c>
       <c r="I2" t="n">
-        <v>92.5</v>
+        <v>90</v>
       </c>
       <c r="J2" t="n">
         <v>25</v>
@@ -9235,47 +9181,47 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>[테마: 사이버보안] 거래량 시그널 60점 (2주avg/4-8주avg = 2.91, 2주/2-4주 = 1.59). 트렌드 시그널 92점 — 매칭 키워드: 사이버보안(naver, 100점), 양자암호(naver, 85점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: 문서·DB 보안</t>
+          <t>[테마: 사이버보안] 거래량 시그널 60점 (2주avg/4-8주avg = 2.91, 2주/2-4주 = 1.59). 트렌드 시그널 90점 — 매칭 키워드: 사이버보안(naver, 100점), 양자암호(naver, 80점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: 문서·DB 보안</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>204270</t>
+          <t>066970</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>제이앤티씨</t>
+          <t>엘앤에프</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>22950</v>
+        <v>120000</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>재생에너지/풍력</t>
+          <t>2차전지/배터리</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>62.8</v>
+        <v>59.5</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>🟡 주목</t>
+          <t>⚪ 관찰</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>60</v>
       </c>
       <c r="I3" t="n">
-        <v>88</v>
+        <v>78.5</v>
       </c>
       <c r="J3" t="n">
         <v>25</v>
@@ -9285,24 +9231,24 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>lioness season 3 how many episodes</t>
+          <t>current events, 분리막</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>[테마: 재생에너지/풍력] 거래량 시그널 60점 (2주avg/4-8주avg = 2.41, 2주/2-4주 = 1.74). 트렌드 시그널 88점 — 매칭 키워드: lioness season 3 how many episodes(google, 88점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: (중복)</t>
+          <t>[테마: 2차전지/배터리] 거래량 시그널 60점 (2주avg/4-8주avg = 2.08, 2주/2-4주 = 1.50). 트렌드 시그널 78점 — 매칭 키워드: current events(google, 96점), 분리막(naver, 45점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: 양극재</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>066970</t>
+          <t>052690</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>엘앤에프</t>
+          <t>한전기술</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -9311,53 +9257,53 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>120000</v>
+        <v>152000</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>데이터센터/AI인프라</t>
+          <t>원전/SMR</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>60.3</v>
+        <v>58.9</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>🟡 주목</t>
+          <t>⚪ 관찰</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>60</v>
       </c>
       <c r="I4" t="n">
-        <v>81</v>
+        <v>62.7</v>
       </c>
       <c r="J4" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="K4" t="b">
         <v>0</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>광통신</t>
+          <t>소형원자로, 원전, 원자력</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>[테마: 데이터센터/AI인프라] 거래량 시그널 60점 (2주avg/4-8주avg = 2.08, 2주/2-4주 = 1.50). 트렌드 시그널 81점 — 매칭 키워드: 광통신(naver, 81점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: (중복)</t>
+          <t>[테마: 원전/SMR] 거래량 시그널 60점 (2주avg/4-8주avg = 5.91, 2주/2-4주 = 1.39). 트렌드 시그널 63점 — 매칭 키워드: 소형원자로(naver, 70점), 원전(naver, 63점), 원자력(naver, 55점). 동일 테마 동시통과 2종목(밀집도 50점). 종목 근거: 원전 설계</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>052690</t>
+          <t>066970</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>한전기술</t>
+          <t>엘앤에프</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -9366,15 +9312,15 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>152000</v>
+        <v>120000</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>원전/SMR</t>
+          <t>데이터센터/AI인프라</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>60</v>
+        <v>58.2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -9385,34 +9331,34 @@
         <v>60</v>
       </c>
       <c r="I5" t="n">
-        <v>65.7</v>
+        <v>75</v>
       </c>
       <c r="J5" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="K5" t="b">
         <v>0</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>소형원자로, 원전, 원자력</t>
+          <t>광통신</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>[테마: 원전/SMR] 거래량 시그널 60점 (2주avg/4-8주avg = 5.91, 2주/2-4주 = 1.39). 트렌드 시그널 66점 — 매칭 키워드: 소형원자로(naver, 71점), 원전(naver, 66점), 원자력(naver, 60점). 동일 테마 동시통과 2종목(밀집도 50점). 종목 근거: 원전 설계</t>
+          <t>[테마: 데이터센터/AI인프라] 거래량 시그널 60점 (2주avg/4-8주avg = 2.08, 2주/2-4주 = 1.50). 트렌드 시그널 75점 — 매칭 키워드: 광통신(naver, 75점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: (중복)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>066970</t>
+          <t>034020</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>엘앤에프</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -9421,15 +9367,15 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>120000</v>
+        <v>90800</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2차전지/배터리</t>
+          <t>원전/SMR</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>58.1</v>
+        <v>50.8</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -9437,80 +9383,25 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>60</v>
+        <v>41.8</v>
       </c>
       <c r="I6" t="n">
-        <v>74.5</v>
+        <v>62.7</v>
       </c>
       <c r="J6" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="K6" t="b">
         <v>0</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>lioness season 3 how many episodes, 분리막</t>
+          <t>소형원자로, 원전, 원자력</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>[테마: 2차전지/배터리] 거래량 시그널 60점 (2주avg/4-8주avg = 2.08, 2주/2-4주 = 1.50). 트렌드 시그널 74점 — 매칭 키워드: lioness season 3 how many episodes(google, 88점), 분리막(naver, 45점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: 양극재</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>034020</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>두산에너빌리티</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>90800</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>원전/SMR</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>51.8</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>⚪ 관찰</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>41.8</v>
-      </c>
-      <c r="I7" t="n">
-        <v>65.7</v>
-      </c>
-      <c r="J7" t="n">
-        <v>50</v>
-      </c>
-      <c r="K7" t="b">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>소형원자로, 원전, 원자력</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>[테마: 원전/SMR] 거래량 시그널 42점 (2주avg/4-8주avg = 1.39, 2주/2-4주 = 1.04). 트렌드 시그널 66점 — 매칭 키워드: 소형원자로(naver, 71점), 원전(naver, 66점), 원자력(naver, 60점). 동일 테마 동시통과 2종목(밀집도 50점). 종목 근거: 원전 주기기</t>
+          <t>[테마: 원전/SMR] 거래량 시그널 42점 (2주avg/4-8주avg = 1.39, 2주/2-4주 = 1.04). 트렌드 시그널 63점 — 매칭 키워드: 소형원자로(naver, 70점), 원전(naver, 63점), 원자력(naver, 55점). 동일 테마 동시통과 2종목(밀집도 50점). 종목 근거: 원전 주기기</t>
         </is>
       </c>
     </row>

</xml_diff>